<commit_message>
Module 5 for Week-01
</commit_message>
<xml_diff>
--- a/week-01/Pour_Judgement_Survey_Results.xlsx
+++ b/week-01/Pour_Judgement_Survey_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/04a19e4a9bb9275a/Desktop/DataAnalytics/week-01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="362" documentId="8_{9B281EA0-B6BE-46F3-B2CB-3BB37D49B48D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60DB517A-04EE-4689-93CC-4D0B17A0EA75}"/>
+  <xr:revisionPtr revIDLastSave="363" documentId="8_{9B281EA0-B6BE-46F3-B2CB-3BB37D49B48D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD6924EF-C54F-46EC-81BD-7B716D854E7F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="141">
   <si>
     <t>ID</t>
   </si>
@@ -482,6 +482,9 @@
   </si>
   <si>
     <t>^ First time!</t>
+  </si>
+  <si>
+    <t>I left above how I checked the cells and the formula I used (did use Copilot to assist)</t>
   </si>
 </sst>
 </file>
@@ -6269,7 +6272,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y48"/>
+  <dimension ref="A1:Y49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
@@ -10716,6 +10719,11 @@
     <row r="48" spans="14:20" x14ac:dyDescent="0.3">
       <c r="N48" t="s">
         <v>128</v>
+      </c>
+    </row>
+    <row r="49" spans="14:14" x14ac:dyDescent="0.3">
+      <c r="N49" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>